<commit_message>
Sync regenerated demo workbook from Eudamed-Upload
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/eudamed_master_data_demo.xlsx
+++ b/templates/eudamed_master_data_demo.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O3"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -437,15 +437,8 @@
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="22" customWidth="1" min="7" max="7"/>
-    <col width="21" customWidth="1" min="8" max="8"/>
-    <col width="21" customWidth="1" min="9" max="9"/>
-    <col width="25" customWidth="1" min="10" max="10"/>
-    <col width="24" customWidth="1" min="11" max="11"/>
-    <col width="14" customWidth="1" min="12" max="12"/>
-    <col width="14" customWidth="1" min="13" max="13"/>
-    <col width="20" customWidth="1" min="14" max="14"/>
-    <col width="14" customWidth="1" min="15" max="15"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -481,47 +474,12 @@
       </c>
       <c r="G1" s="2" t="inlineStr">
         <is>
-          <t>animal_tissues_cells</t>
+          <t>active</t>
         </is>
       </c>
       <c r="H1" s="2" t="inlineStr">
         <is>
-          <t>human_tissues_cells</t>
-        </is>
-      </c>
-      <c r="I1" s="2" t="inlineStr">
-        <is>
-          <t>human_product_check</t>
-        </is>
-      </c>
-      <c r="J1" s="2" t="inlineStr">
-        <is>
-          <t>medicinal_product_check</t>
-        </is>
-      </c>
-      <c r="K1" s="2" t="inlineStr">
-        <is>
-          <t>administering_medicine</t>
-        </is>
-      </c>
-      <c r="L1" s="2" t="inlineStr">
-        <is>
-          <t>active</t>
-        </is>
-      </c>
-      <c r="M1" s="2" t="inlineStr">
-        <is>
-          <t>implantable</t>
-        </is>
-      </c>
-      <c r="N1" s="2" t="inlineStr">
-        <is>
           <t>measuring_function</t>
-        </is>
-      </c>
-      <c r="O1" s="2" t="inlineStr">
-        <is>
-          <t>reusable</t>
         </is>
       </c>
     </row>
@@ -566,41 +524,6 @@
           <t>FALSE</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -635,52 +558,17 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>FALSE</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
           <t>TRUE</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
     </row>
   </sheetData>
-  <dataValidations count="12">
+  <dataValidations count="5">
     <dataValidation sqref="B2:B201" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list">
       <formula1>"EUDAMED,GS1,HIBCC,ICCBBA,IFA"</formula1>
     </dataValidation>
@@ -694,27 +582,6 @@
       <formula1>"TRUE,FALSE"</formula1>
     </dataValidation>
     <dataValidation sqref="H2:H201" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
-      <formula1>"TRUE,FALSE"</formula1>
-    </dataValidation>
-    <dataValidation sqref="I2:I201" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
-      <formula1>"TRUE,FALSE"</formula1>
-    </dataValidation>
-    <dataValidation sqref="J2:J201" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
-      <formula1>"TRUE,FALSE"</formula1>
-    </dataValidation>
-    <dataValidation sqref="K2:K201" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
-      <formula1>"TRUE,FALSE"</formula1>
-    </dataValidation>
-    <dataValidation sqref="L2:L201" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
-      <formula1>"TRUE,FALSE"</formula1>
-    </dataValidation>
-    <dataValidation sqref="M2:M201" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
-      <formula1>"TRUE,FALSE"</formula1>
-    </dataValidation>
-    <dataValidation sqref="N2:N201" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
-      <formula1>"TRUE,FALSE"</formula1>
-    </dataValidation>
-    <dataValidation sqref="O2:O201" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"TRUE,FALSE"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>